<commit_message>
new accepted and submitted
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A54D254-A5BA-488B-A690-06BBE2E3AD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13186BAF-33A1-411A-8A28-F0751E314714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,12 +28,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3644" uniqueCount="1543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3731" uniqueCount="1564">
   <si>
     <t>title</t>
   </si>
@@ -4430,9 +4433,6 @@
     <t>De Pauw, Robby; Lakha, Fatim; Fletcher, Eilidh; Stockton, Diane L; Baird, Emma; Connolly, Suzanne; Devleesschauwer, Brecht; Wyper, Grant M A</t>
   </si>
   <si>
-    <t>10.1101/2025.01.07.24319409</t>
-  </si>
-  <si>
     <t>e70487</t>
   </si>
   <si>
@@ -4625,9 +4625,6 @@
     <t>10.1186/s13690-025-01652-x</t>
   </si>
   <si>
-    <t>10.21203/rs.3.rs-5611920/v1</t>
-  </si>
-  <si>
     <t>Pre-pandemic sub-national disparities in the disease burden of ischemic heart disease and stroke in France</t>
   </si>
   <si>
@@ -4662,6 +4659,75 @@
   </si>
   <si>
     <t>Couchoud, Cécile; Raffray, Maxime; Mahrouseh, Nour; von der Lippe, Elena; Devleesschauwer, Brecht; Wyper, Grant M A; Haneef, Romana</t>
+  </si>
+  <si>
+    <t>10.1016/j.actatropica.2025.107828</t>
+  </si>
+  <si>
+    <t>10.1186/s12874-025-02661-8</t>
+  </si>
+  <si>
+    <t>Social inequalities in COVID-19-related years of life lost in metropolitan France, 2020</t>
+  </si>
+  <si>
+    <t>Haneef, Romana; Mahrouseh, Nour; Bessonneau, P; Vandentorren, Stephanie; Minier, N; Chin, F; Bruyère, Olivier; Devleesschauwer, Brecht; Wyper, Grant M A</t>
+  </si>
+  <si>
+    <t>10.1186/s13690-025-01704-2</t>
+  </si>
+  <si>
+    <t>Past trends, future forecasts and socio-demographic patterns of cigarette smoking in Belgium, 1997 to 2040</t>
+  </si>
+  <si>
+    <t>10.1186/s13690-025-01694-1</t>
+  </si>
+  <si>
+    <t>10.1016/j.puhe.2025.105981</t>
+  </si>
+  <si>
+    <t>10.1093/eurpub/ckaf190</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10.1186/s13690-025-01767-1 </t>
+  </si>
+  <si>
+    <t>Subtype-specific health and economic impact of delayed breast cancer diagnosis during the early COVID-19 pandemic in Belgium: a Markov model analysis</t>
+  </si>
+  <si>
+    <t>10.1186/s13058-025-02207-2</t>
+  </si>
+  <si>
+    <t>Breast Cancer Res.</t>
+  </si>
+  <si>
+    <t>Breast Cancer Research</t>
+  </si>
+  <si>
+    <t>Khan, Yasmine; Verhaeghe, Nick; Monten, Chris; Vanthomme, Katrien; Gadeyne, Sylvie; Devleesschauwer, Brecht; Verdoodt, Freija; Peacock, Hanna M; De Smedt, Delphine</t>
+  </si>
+  <si>
+    <t>Social inequalities in in-hospital mortality following COVID-19 hospitalization in Belgium: a competing risk survival analysis</t>
+  </si>
+  <si>
+    <t>BMC Health Services Research</t>
+  </si>
+  <si>
+    <t>BMC Health. Serv. Res.</t>
+  </si>
+  <si>
+    <t>Social inequalities in cause-specific premature mortality in rural and urban areas of mainland France using population attributable fractions (PAFs): a pre-pandemic analysis</t>
+  </si>
+  <si>
+    <t>Mahrouseh, Nour; Bonnet, Florian; Varga, Orsolya; Scohy, Aline; Bruyère, Olivier; Delpierre, Cyrille; Devleesschauwer, Brecht; Wyper, Grant M A;  Haneef, Romana</t>
+  </si>
+  <si>
+    <t>Boiy, Elin; Cavillot, Lisa; Devleesschauwer, Brecht; De Smedt, Delphine; Gadeyne, Sylvie; Speybroeck, Niko; Van den Borre, Laura; Vanthomme, Katrien; Verhaege, Nick; De Pauw, Robby</t>
+  </si>
+  <si>
+    <t>World Health Organization estimates of the global, regional, and national burden of seven foodborne bacterial and viral invasive enteric diseases and one foodborne intoxication, 2000-2021: an updated data synthesis</t>
+  </si>
+  <si>
+    <t>Majowicz, Shannon E; Scallan Walter, Elaine; Pires, Sara M; Minato, Yuki; Founou, Luria; Devleesschauwer, Brecht; Di Bari, Carlotta; Havelaar, Arie H; Vaes, Louise; Estrada Garcia, Teresa; Roberts, Charlee; Gobena, Tesfaye; Kumar, Ashok; Al Natour, Fadi; Lake, Robin J; Nane, Gabriela F; Fernandez, Kim; Crump, John A; Kirk, Martyn D</t>
   </si>
 </sst>
 </file>
@@ -5083,6 +5149,82 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="165" formatCode="0.0"/>
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -5170,82 +5312,6 @@
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
@@ -5260,74 +5326,74 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabel1" displayName="Tabel1" ref="A1:U279" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
-  <autoFilter ref="A1:U279" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U279">
-    <sortCondition ref="K1:K279"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabel1" displayName="Tabel1" ref="A1:U288" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+  <autoFilter ref="A1:U288" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U286">
+    <sortCondition ref="K1:K286"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="title" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="authors" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="journal_full" dataDxfId="59"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="journal_short" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="year" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="volume" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="issue" dataDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="eID" dataDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="from" dataDxfId="53"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="to" dataDxfId="52"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="date" dataDxfId="51"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="date_submitted" dataDxfId="50" dataCellStyle="Neutral"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="classification" dataDxfId="49"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="IF" dataDxfId="48"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DOI" dataDxfId="47"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="WoS" dataDxfId="46"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="rank" dataDxfId="45"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="quartile" dataDxfId="44"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="category" dataDxfId="43"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="SC" dataDxfId="42"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="UGent" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="title" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="authors" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="journal_full" dataDxfId="31"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="journal_short" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="year" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="volume" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="issue" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="eID" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="from" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="to" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="date" dataDxfId="23"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="date_submitted" dataDxfId="22" dataCellStyle="Neutral"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="classification" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="IF" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="DOI" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="WoS" dataDxfId="18"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="rank" dataDxfId="17"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="quartile" dataDxfId="16"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="category" dataDxfId="15"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="SC" dataDxfId="14"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="UGent" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabel14" displayName="Tabel14" ref="A1:J12" totalsRowShown="0" headerRowDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabel14" displayName="Tabel14" ref="A1:J12" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="A1:J12" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N50">
     <sortCondition ref="H1:H50"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="title" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="authors" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="editors" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="book" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="year" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="from" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="to" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="date" dataDxfId="32"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="IF" dataDxfId="31"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="DOI" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="title" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="authors" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="editors" dataDxfId="60"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="book" dataDxfId="59"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="year" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="from" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="to" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="date" dataDxfId="55"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="IF" dataDxfId="54"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="DOI" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabel13" displayName="Tabel13" ref="A1:G22" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
-  <autoFilter ref="A1:G22" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G17">
-    <sortCondition ref="F1:F17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabel13" displayName="Tabel13" ref="A1:G19" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+  <autoFilter ref="A1:G19" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G16">
+    <sortCondition ref="F1:F16"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="title" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="authors" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="journal_full" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="journal_short" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="doi_preprint" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="date" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="COUNT" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="title" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="authors" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="journal_full" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="journal_short" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="doi_preprint" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="date" dataDxfId="45"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="COUNT" dataDxfId="44">
       <calculatedColumnFormula>TODAY()-F2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5336,18 +5402,18 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabel135" displayName="Tabel135" ref="A1:F5" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabel135" displayName="Tabel135" ref="A1:F5" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="A1:F5" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K14">
     <sortCondition ref="E1:E14"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="title" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="authors" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="journal_full" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="journal_short" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="date" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="COUNT" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="title" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="authors" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="journal_full" dataDxfId="39"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="journal_short" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="date" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="COUNT" dataDxfId="36">
       <calculatedColumnFormula>(TODAY()-E2)/365</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5676,7 +5742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U279"/>
+  <dimension ref="A1:U288"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -19924,7 +19990,7 @@
     </row>
     <row r="263" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A263" s="7" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="B263" s="7" t="s">
         <v>1213</v>
@@ -19945,7 +20011,7 @@
         <v>14</v>
       </c>
       <c r="H263" s="18" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="I263" s="18" t="s">
         <v>14</v>
@@ -19962,14 +20028,16 @@
       </c>
       <c r="N263" s="11"/>
       <c r="O263" s="19" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="P263" s="7"/>
       <c r="Q263" s="24"/>
       <c r="R263" s="25"/>
       <c r="S263" s="7"/>
       <c r="T263" s="7"/>
-      <c r="U263" s="7"/>
+      <c r="U263" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="264" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A264" s="7" t="s">
@@ -20047,7 +20115,7 @@
         <v>101</v>
       </c>
       <c r="H265" s="18" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="I265" s="18" t="s">
         <v>14</v>
@@ -20064,27 +20132,29 @@
       </c>
       <c r="N265" s="11"/>
       <c r="O265" s="19" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="P265" s="7"/>
       <c r="Q265" s="24"/>
       <c r="R265" s="25"/>
       <c r="S265" s="7"/>
       <c r="T265" s="7"/>
-      <c r="U265" s="7"/>
+      <c r="U265" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="266" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A266" s="7" t="s">
+        <v>1487</v>
+      </c>
+      <c r="B266" s="7" t="s">
         <v>1488</v>
-      </c>
-      <c r="B266" s="7" t="s">
-        <v>1489</v>
       </c>
       <c r="C266" s="7" t="s">
         <v>267</v>
       </c>
       <c r="D266" s="7" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
       <c r="E266" s="18">
         <v>2025</v>
@@ -20113,14 +20183,16 @@
       </c>
       <c r="N266" s="11"/>
       <c r="O266" s="19" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
       <c r="P266" s="7"/>
       <c r="Q266" s="24"/>
       <c r="R266" s="25"/>
       <c r="S266" s="7"/>
       <c r="T266" s="7"/>
-      <c r="U266" s="7"/>
+      <c r="U266" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="267" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A267" s="7" t="s">
@@ -20162,18 +20234,20 @@
       </c>
       <c r="N267" s="11"/>
       <c r="O267" s="19" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="P267" s="7"/>
       <c r="Q267" s="24"/>
       <c r="R267" s="25"/>
       <c r="S267" s="7"/>
       <c r="T267" s="7"/>
-      <c r="U267" s="7"/>
+      <c r="U267" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="268" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A268" s="7" t="s">
-        <v>1518</v>
+        <v>1517</v>
       </c>
       <c r="B268" s="7" t="s">
         <v>1260</v>
@@ -20211,27 +20285,29 @@
       </c>
       <c r="N268" s="11"/>
       <c r="O268" s="19" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
       <c r="P268" s="7"/>
       <c r="Q268" s="24"/>
       <c r="R268" s="25"/>
       <c r="S268" s="7"/>
       <c r="T268" s="7"/>
-      <c r="U268" s="7"/>
+      <c r="U268" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="269" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A269" s="7" t="s">
+        <v>1479</v>
+      </c>
+      <c r="B269" s="7" t="s">
         <v>1480</v>
       </c>
-      <c r="B269" s="7" t="s">
+      <c r="C269" s="7" t="s">
         <v>1481</v>
       </c>
-      <c r="C269" s="7" t="s">
+      <c r="D269" s="7" t="s">
         <v>1482</v>
-      </c>
-      <c r="D269" s="7" t="s">
-        <v>1483</v>
       </c>
       <c r="E269" s="18">
         <v>2025</v>
@@ -20246,10 +20322,10 @@
         <v>14</v>
       </c>
       <c r="I269" s="18" t="s">
+        <v>1483</v>
+      </c>
+      <c r="J269" s="18" t="s">
         <v>1484</v>
-      </c>
-      <c r="J269" s="18" t="s">
-        <v>1485</v>
       </c>
       <c r="K269" s="42">
         <v>45706</v>
@@ -20260,21 +20336,23 @@
       </c>
       <c r="N269" s="11"/>
       <c r="O269" s="19" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="P269" s="7"/>
       <c r="Q269" s="24"/>
       <c r="R269" s="25"/>
       <c r="S269" s="7"/>
       <c r="T269" s="7"/>
-      <c r="U269" s="7"/>
+      <c r="U269" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="270" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A270" s="7" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
       <c r="B270" s="7" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="C270" s="7" t="s">
         <v>723</v>
@@ -20292,7 +20370,7 @@
         <v>548</v>
       </c>
       <c r="H270" s="18" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
       <c r="I270" s="18" t="s">
         <v>14</v>
@@ -20309,21 +20387,23 @@
       </c>
       <c r="N270" s="11"/>
       <c r="O270" s="19" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="P270" s="7"/>
       <c r="Q270" s="24"/>
       <c r="R270" s="25"/>
       <c r="S270" s="7"/>
       <c r="T270" s="7"/>
-      <c r="U270" s="7"/>
+      <c r="U270" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="271" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A271" s="7" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="B271" s="7" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="C271" s="7" t="s">
         <v>373</v>
@@ -20358,14 +20438,16 @@
       </c>
       <c r="N271" s="11"/>
       <c r="O271" s="19" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="P271" s="7"/>
       <c r="Q271" s="24"/>
       <c r="R271" s="25"/>
       <c r="S271" s="7"/>
       <c r="T271" s="7"/>
-      <c r="U271" s="7"/>
+      <c r="U271" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="272" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A272" s="7" t="s">
@@ -20390,7 +20472,7 @@
         <v>548</v>
       </c>
       <c r="H272" s="18" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="I272" s="18" t="s">
         <v>14</v>
@@ -20407,27 +20489,29 @@
       </c>
       <c r="N272" s="11"/>
       <c r="O272" s="19" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="P272" s="7"/>
       <c r="Q272" s="24"/>
       <c r="R272" s="25"/>
       <c r="S272" s="7"/>
       <c r="T272" s="7"/>
-      <c r="U272" s="7"/>
+      <c r="U272" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="273" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A273" s="7" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
       <c r="B273" s="7" t="s">
         <v>1316</v>
       </c>
       <c r="C273" s="7" t="s">
+        <v>1499</v>
+      </c>
+      <c r="D273" s="7" t="s">
         <v>1500</v>
-      </c>
-      <c r="D273" s="7" t="s">
-        <v>1501</v>
       </c>
       <c r="E273" s="18">
         <v>2025</v>
@@ -20456,21 +20540,23 @@
       </c>
       <c r="N273" s="11"/>
       <c r="O273" s="19" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
       <c r="P273" s="7"/>
       <c r="Q273" s="24"/>
       <c r="R273" s="25"/>
       <c r="S273" s="7"/>
       <c r="T273" s="7"/>
-      <c r="U273" s="7"/>
+      <c r="U273" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="274" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A274" s="7" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="B274" s="7" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="C274" s="7" t="s">
         <v>723</v>
@@ -20488,7 +20574,7 @@
         <v>111</v>
       </c>
       <c r="H274" s="18" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
       <c r="I274" s="18" t="s">
         <v>14</v>
@@ -20505,21 +20591,23 @@
       </c>
       <c r="N274" s="11"/>
       <c r="O274" s="19" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
       <c r="P274" s="7"/>
       <c r="Q274" s="24"/>
       <c r="R274" s="25"/>
       <c r="S274" s="7"/>
       <c r="T274" s="7"/>
-      <c r="U274" s="7"/>
+      <c r="U274" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="275" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A275" s="7" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="B275" s="7" t="s">
-        <v>1527</v>
+        <v>1526</v>
       </c>
       <c r="C275" s="7" t="s">
         <v>89</v>
@@ -20554,21 +20642,23 @@
       </c>
       <c r="N275" s="11"/>
       <c r="O275" s="19" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="P275" s="7"/>
       <c r="Q275" s="24"/>
       <c r="R275" s="25"/>
       <c r="S275" s="7"/>
       <c r="T275" s="7"/>
-      <c r="U275" s="7"/>
+      <c r="U275" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="276" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A276" s="7" t="s">
+        <v>1493</v>
+      </c>
+      <c r="B276" s="7" t="s">
         <v>1494</v>
-      </c>
-      <c r="B276" s="7" t="s">
-        <v>1495</v>
       </c>
       <c r="C276" s="7" t="s">
         <v>267</v>
@@ -20603,14 +20693,16 @@
       </c>
       <c r="N276" s="11"/>
       <c r="O276" s="19" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="P276" s="7"/>
       <c r="Q276" s="24"/>
       <c r="R276" s="25"/>
       <c r="S276" s="7"/>
       <c r="T276" s="7"/>
-      <c r="U276" s="7"/>
+      <c r="U276" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="277" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A277" s="7" t="s">
@@ -20652,21 +20744,23 @@
       </c>
       <c r="N277" s="11"/>
       <c r="O277" s="19" t="s">
-        <v>1526</v>
+        <v>1525</v>
       </c>
       <c r="P277" s="7"/>
       <c r="Q277" s="24"/>
       <c r="R277" s="25"/>
       <c r="S277" s="7"/>
       <c r="T277" s="7"/>
-      <c r="U277" s="7"/>
+      <c r="U277" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="278" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A278" s="7" t="s">
         <v>1346</v>
       </c>
       <c r="B278" s="7" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="C278" s="7" t="s">
         <v>160</v>
@@ -20684,7 +20778,7 @@
         <v>153</v>
       </c>
       <c r="H278" s="18" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="I278" s="18" t="s">
         <v>14</v>
@@ -20701,66 +20795,513 @@
       </c>
       <c r="N278" s="11"/>
       <c r="O278" s="19" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="P278" s="7"/>
       <c r="Q278" s="24"/>
       <c r="R278" s="25"/>
       <c r="S278" s="7"/>
       <c r="T278" s="7"/>
-      <c r="U278" s="7"/>
+      <c r="U278" s="7" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="279" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A279" s="13" t="s">
-        <v>1093</v>
-      </c>
-      <c r="B279" s="13" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C279" s="13" t="s">
-        <v>1095</v>
-      </c>
-      <c r="D279" s="13" t="s">
-        <v>1096</v>
-      </c>
-      <c r="E279" s="14">
+      <c r="A279" s="7" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B279" s="7" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C279" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D279" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="E279" s="18">
         <v>2025</v>
       </c>
-      <c r="F279" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="G279" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="H279" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="I279" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="J279" s="43" t="s">
-        <v>14</v>
-      </c>
-      <c r="K279" s="31">
-        <v>46023</v>
-      </c>
-      <c r="L279" s="31"/>
-      <c r="M279" s="31" t="s">
-        <v>273</v>
-      </c>
-      <c r="N279" s="45"/>
-      <c r="O279" s="44" t="s">
-        <v>1264</v>
-      </c>
-      <c r="P279" s="27"/>
+      <c r="F279" s="18">
+        <v>83</v>
+      </c>
+      <c r="G279" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H279" s="18">
+        <v>215</v>
+      </c>
+      <c r="I279" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J279" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K279" s="42">
+        <v>45891</v>
+      </c>
+      <c r="L279" s="42"/>
+      <c r="M279" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N279" s="11"/>
+      <c r="O279" s="19" t="s">
+        <v>1545</v>
+      </c>
+      <c r="P279" s="7"/>
       <c r="Q279" s="24"/>
       <c r="R279" s="25"/>
       <c r="S279" s="7"/>
       <c r="T279" s="7"/>
-      <c r="U279" s="7"/>
+      <c r="U279" s="7" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="280" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A280" s="7" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B280" s="7" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C280" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="D280" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="E280" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F280" s="18">
+        <v>25</v>
+      </c>
+      <c r="G280" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H280" s="18">
+        <v>209</v>
+      </c>
+      <c r="I280" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J280" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K280" s="42">
+        <v>45902</v>
+      </c>
+      <c r="L280" s="42"/>
+      <c r="M280" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N280" s="11"/>
+      <c r="O280" s="19" t="s">
+        <v>1542</v>
+      </c>
+      <c r="P280" s="7"/>
+      <c r="Q280" s="24"/>
+      <c r="R280" s="25"/>
+      <c r="S280" s="7"/>
+      <c r="T280" s="7"/>
+      <c r="U280" s="7" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="281" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A281" s="7" t="s">
+        <v>1496</v>
+      </c>
+      <c r="B281" s="7" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C281" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D281" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E281" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F281" s="18">
+        <v>270</v>
+      </c>
+      <c r="G281" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H281" s="18">
+        <v>107828</v>
+      </c>
+      <c r="I281" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J281" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K281" s="42">
+        <v>45931</v>
+      </c>
+      <c r="L281" s="42"/>
+      <c r="M281" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N281" s="11"/>
+      <c r="O281" s="19" t="s">
+        <v>1541</v>
+      </c>
+      <c r="P281" s="7"/>
+      <c r="Q281" s="24"/>
+      <c r="R281" s="25"/>
+      <c r="S281" s="7"/>
+      <c r="T281" s="7"/>
+      <c r="U281" s="7" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="282" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A282" s="7" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B282" s="7" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C282" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D282" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="E282" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F282" s="18">
+        <v>83</v>
+      </c>
+      <c r="G282" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H282" s="18">
+        <v>256</v>
+      </c>
+      <c r="I282" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J282" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K282" s="42">
+        <v>45953</v>
+      </c>
+      <c r="L282" s="42"/>
+      <c r="M282" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N282" s="11"/>
+      <c r="O282" s="19" t="s">
+        <v>1547</v>
+      </c>
+      <c r="P282" s="7"/>
+      <c r="Q282" s="24"/>
+      <c r="R282" s="25"/>
+      <c r="S282" s="7"/>
+      <c r="T282" s="7"/>
+      <c r="U282" s="7"/>
+    </row>
+    <row r="283" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A283" s="7" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B283" s="7" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C283" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D283" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="E283" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F283" s="18">
+        <v>35</v>
+      </c>
+      <c r="G283" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="H283" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I283" s="18">
+        <v>1122</v>
+      </c>
+      <c r="J283" s="18">
+        <v>1128</v>
+      </c>
+      <c r="K283" s="42">
+        <v>45960</v>
+      </c>
+      <c r="L283" s="42"/>
+      <c r="M283" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N283" s="11"/>
+      <c r="O283" s="19" t="s">
+        <v>1549</v>
+      </c>
+      <c r="P283" s="7"/>
+      <c r="Q283" s="24"/>
+      <c r="R283" s="25"/>
+      <c r="S283" s="7"/>
+      <c r="T283" s="7"/>
+      <c r="U283" s="7"/>
+    </row>
+    <row r="284" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A284" s="7" t="s">
+        <v>1463</v>
+      </c>
+      <c r="B284" s="7" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C284" s="7" t="s">
+        <v>1462</v>
+      </c>
+      <c r="D284" s="7" t="s">
+        <v>1462</v>
+      </c>
+      <c r="E284" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F284" s="18">
+        <v>248</v>
+      </c>
+      <c r="G284" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H284" s="18">
+        <v>105981</v>
+      </c>
+      <c r="I284" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J284" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K284" s="42">
+        <v>45962</v>
+      </c>
+      <c r="L284" s="42"/>
+      <c r="M284" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N284" s="11"/>
+      <c r="O284" s="19" t="s">
+        <v>1548</v>
+      </c>
+      <c r="P284" s="7"/>
+      <c r="Q284" s="24"/>
+      <c r="R284" s="25"/>
+      <c r="S284" s="7"/>
+      <c r="T284" s="7"/>
+      <c r="U284" s="7"/>
+    </row>
+    <row r="285" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A285" s="7" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B285" s="7" t="s">
+        <v>1540</v>
+      </c>
+      <c r="C285" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D285" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="E285" s="18">
+        <v>2025</v>
+      </c>
+      <c r="F285" s="18">
+        <v>83</v>
+      </c>
+      <c r="G285" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H285" s="18">
+        <v>298</v>
+      </c>
+      <c r="I285" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J285" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K285" s="42">
+        <v>46001</v>
+      </c>
+      <c r="L285" s="42"/>
+      <c r="M285" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="N285" s="11"/>
+      <c r="O285" s="19" t="s">
+        <v>1550</v>
+      </c>
+      <c r="P285" s="7"/>
+      <c r="Q285" s="24"/>
+      <c r="R285" s="25"/>
+      <c r="S285" s="7"/>
+      <c r="T285" s="7"/>
+      <c r="U285" s="7"/>
+    </row>
+    <row r="286" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A286" s="13" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B286" s="13" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C286" s="13" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D286" s="13" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E286" s="14">
+        <v>2026</v>
+      </c>
+      <c r="F286" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G286" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="H286" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="I286" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="J286" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="K286" s="31">
+        <v>46023</v>
+      </c>
+      <c r="L286" s="31"/>
+      <c r="M286" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="N286" s="45"/>
+      <c r="O286" s="44" t="s">
+        <v>1264</v>
+      </c>
+      <c r="P286" s="27"/>
+      <c r="Q286" s="24"/>
+      <c r="R286" s="25"/>
+      <c r="S286" s="7"/>
+      <c r="T286" s="7"/>
+      <c r="U286" s="7"/>
+    </row>
+    <row r="287" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A287" s="13" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B287" s="13" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C287" s="13" t="s">
+        <v>1554</v>
+      </c>
+      <c r="D287" s="13" t="s">
+        <v>1553</v>
+      </c>
+      <c r="E287" s="14">
+        <v>2026</v>
+      </c>
+      <c r="F287" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G287" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="H287" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="I287" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="J287" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="K287" s="31">
+        <v>46024</v>
+      </c>
+      <c r="L287" s="31"/>
+      <c r="M287" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="N287" s="45"/>
+      <c r="O287" s="44" t="s">
+        <v>1552</v>
+      </c>
+      <c r="P287" s="27"/>
+      <c r="Q287" s="24"/>
+      <c r="R287" s="25"/>
+      <c r="S287" s="7"/>
+      <c r="T287" s="7"/>
+      <c r="U287" s="7"/>
+    </row>
+    <row r="288" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A288" s="13" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B288" s="13" t="s">
+        <v>1320</v>
+      </c>
+      <c r="C288" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D288" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="E288" s="14">
+        <v>2026</v>
+      </c>
+      <c r="F288" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G288" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="H288" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="I288" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="J288" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="K288" s="31">
+        <v>46025</v>
+      </c>
+      <c r="L288" s="31"/>
+      <c r="M288" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="N288" s="45"/>
+      <c r="O288" s="44"/>
+      <c r="P288" s="27"/>
+      <c r="Q288" s="24"/>
+      <c r="R288" s="25"/>
+      <c r="S288" s="7"/>
+      <c r="T288" s="7"/>
+      <c r="U288" s="7"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="T1:U112 T114:U231 V246:V247 T232:V240 V241:V242 T241:T242 T248:V1048576 T243:V245 T246:U246">
+  <conditionalFormatting sqref="T1:U112 T114:U231 V246:V247 T232:V240 V241:V242 T241:T242 T243:V245 T246:U246 T248:V1048576">
     <cfRule type="cellIs" dxfId="12" priority="31" operator="equal">
       <formula>"N/A"</formula>
     </cfRule>
@@ -21187,7 +21728,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="40.7109375" customWidth="1"/>
@@ -21221,11 +21762,11 @@
       </c>
       <c r="I1" s="55" t="str">
         <f ca="1">ROUND(J1/30,0)&amp;" md"</f>
-        <v>5 md</v>
+        <v>8 md</v>
       </c>
       <c r="J1" s="55">
         <f ca="1">AVERAGE(G:G)</f>
-        <v>145.14285714285714</v>
+        <v>237.88888888888889</v>
       </c>
       <c r="K1" s="54" t="s">
         <v>1164</v>
@@ -21249,8 +21790,8 @@
         <v>45488</v>
       </c>
       <c r="G2" s="12">
-        <f t="shared" ref="G2:G22" ca="1" si="0">TODAY()-F2</f>
-        <v>375</v>
+        <f t="shared" ref="G2:G19" ca="1" si="0">TODAY()-F2</f>
+        <v>535</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -21272,7 +21813,7 @@
       </c>
       <c r="G3" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>339</v>
+        <v>499</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -21294,7 +21835,7 @@
       </c>
       <c r="G4" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>301</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -21316,385 +21857,315 @@
       </c>
       <c r="G5" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>239</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>1454</v>
+        <v>1314</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>89</v>
+        <v>723</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>89</v>
+        <v>723</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="10">
-        <v>45624</v>
+        <v>45705</v>
       </c>
       <c r="G6" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>239</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>1450</v>
+        <v>1475</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>1451</v>
+        <v>1476</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>267</v>
+        <v>1477</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>1530</v>
-      </c>
+        <v>1478</v>
+      </c>
+      <c r="E7" s="7"/>
       <c r="F7" s="10">
-        <v>45636</v>
+        <v>45729</v>
       </c>
       <c r="G7" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>227</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>1448</v>
+        <v>1510</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>1449</v>
+        <v>1512</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>668</v>
+        <v>89</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>669</v>
+        <v>89</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="10">
-        <v>45637</v>
+        <v>45764</v>
       </c>
       <c r="G8" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>226</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>1463</v>
+        <v>1514</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>1464</v>
+        <v>1516</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>1462</v>
+        <v>1111</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>1462</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>1465</v>
-      </c>
+        <v>1112</v>
+      </c>
+      <c r="E9" s="7"/>
       <c r="F9" s="10">
-        <v>45663</v>
+        <v>45790</v>
       </c>
       <c r="G9" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>200</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>1469</v>
+        <v>1513</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>1470</v>
+        <v>1515</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>287</v>
+        <v>1557</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>330</v>
+        <v>1558</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="10">
-        <v>45671</v>
+        <v>45803</v>
       </c>
       <c r="G10" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>192</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>1314</v>
+        <v>1537</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>1318</v>
+        <v>1538</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>723</v>
+        <v>89</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>723</v>
+        <v>89</v>
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="10">
-        <v>45705</v>
+        <v>45845</v>
       </c>
       <c r="G11" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>158</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>1476</v>
+        <v>1508</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>1477</v>
+        <v>1509</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>1478</v>
+        <v>108</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>1479</v>
+        <v>109</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="10">
-        <v>45729</v>
+        <v>45853</v>
       </c>
       <c r="G12" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>134</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>1497</v>
+        <v>1529</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>1498</v>
+        <v>1530</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>160</v>
+        <v>1531</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>1313</v>
+        <v>1532</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="10">
-        <v>45735</v>
+        <v>45854</v>
       </c>
       <c r="G13" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>128</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>1511</v>
+        <v>1533</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>1513</v>
+        <v>1539</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>89</v>
+        <v>1024</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>89</v>
+        <v>1026</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="10">
-        <v>45764</v>
+        <v>45860</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>1509</v>
+        <v>1534</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>1510</v>
+        <v>1535</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>108</v>
+        <v>1024</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>109</v>
+        <v>1026</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="10">
-        <v>45853</v>
+        <v>45860</v>
       </c>
       <c r="G15" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>1515</v>
+        <v>1546</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>1517</v>
+        <v>1512</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>1111</v>
+        <v>108</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>1112</v>
+        <v>109</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="10">
-        <v>45790</v>
+        <v>45896</v>
       </c>
       <c r="G16" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>1514</v>
+        <v>1559</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>1516</v>
+        <v>1560</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>1111</v>
+        <v>108</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>1112</v>
+        <v>109</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="10">
-        <v>45803</v>
+        <v>46008</v>
       </c>
       <c r="G17" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>1531</v>
+        <v>1556</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>1532</v>
+        <v>1561</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>1533</v>
+        <v>1462</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>1534</v>
+        <v>1462</v>
       </c>
       <c r="E18" s="7"/>
       <c r="F18" s="10">
-        <v>45854</v>
+        <v>45944</v>
       </c>
       <c r="G18" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>1535</v>
+        <v>1562</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>1541</v>
+        <v>1563</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>1024</v>
+        <v>120</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>1026</v>
+        <v>121</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="10">
-        <v>45860</v>
+        <v>46023</v>
       </c>
       <c r="G19" s="12">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>1536</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>1537</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>1024</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>1026</v>
-      </c>
-      <c r="E20" s="7"/>
-      <c r="F20" s="10">
-        <v>45860</v>
-      </c>
-      <c r="G20" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>1538</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>1542</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="10">
-        <v>45848</v>
-      </c>
-      <c r="G21" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>1539</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>1540</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="10">
-        <v>45845</v>
-      </c>
-      <c r="G22" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -21756,7 +22227,7 @@
       </c>
       <c r="F2" s="40">
         <f t="shared" ref="F2:F4" ca="1" si="0">(TODAY()-E2)/365</f>
-        <v>9.7397260273972606</v>
+        <v>10.178082191780822</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -21777,7 +22248,7 @@
       </c>
       <c r="F3" s="40">
         <f t="shared" ca="1" si="0"/>
-        <v>9.7397260273972606</v>
+        <v>10.178082191780822</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -21798,7 +22269,7 @@
       </c>
       <c r="F4" s="40">
         <f t="shared" ca="1" si="0"/>
-        <v>9.117808219178082</v>
+        <v>9.5561643835616437</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -21819,7 +22290,7 @@
       </c>
       <c r="F5" s="40">
         <f ca="1">(TODAY()-E5)/365</f>
-        <v>7.4876712328767123</v>
+        <v>7.9260273972602739</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -23350,13 +23821,13 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="B74" s="15">
         <v>2025</v>
       </c>
       <c r="C74" s="49" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="E74" s="15" t="s">
         <v>1044</v>

</xml_diff>